<commit_message>
Merge team automation modules
</commit_message>
<xml_diff>
--- a/testData/Testdata.xlsx
+++ b/testData/Testdata.xlsx
@@ -5,19 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\asumi\LMS_PLAYWRIGHTPROJECT\testData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c5ca9bbbfa311c03/Documents/LMS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5AF0033-6383-45AA-8D2B-ED40FA8C7055}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{D5AF0033-6383-45AA-8D2B-ED40FA8C7055}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{685B5F6E-B3C8-4840-B48F-2F972F45AEAE}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
-    <sheet name="Home" sheetId="2" r:id="rId2"/>
-    <sheet name="Program" sheetId="3" r:id="rId3"/>
-    <sheet name="Batch" sheetId="4" r:id="rId4"/>
-    <sheet name="Logout" sheetId="5" r:id="rId5"/>
+    <sheet name="Program" sheetId="3" r:id="rId2"/>
+    <sheet name="Batch" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -29,16 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="22">
-  <si>
-    <t>Test Sceanrio Id</t>
-  </si>
-  <si>
-    <t>Sceanrio Name</t>
-  </si>
-  <si>
-    <t>Username</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="72">
   <si>
     <t>Password</t>
   </si>
@@ -46,27 +35,12 @@
     <t>Result</t>
   </si>
   <si>
-    <t>Scenario Name</t>
-  </si>
-  <si>
-    <t>Test ScenarioID</t>
-  </si>
-  <si>
     <t>ProgramName</t>
   </si>
   <si>
-    <t>ProgramDescription</t>
-  </si>
-  <si>
     <t>Status</t>
   </si>
   <si>
-    <t>Menu</t>
-  </si>
-  <si>
-    <t>Visible</t>
-  </si>
-  <si>
     <t>CypressLMSApplication</t>
   </si>
   <si>
@@ -95,13 +69,187 @@
   </si>
   <si>
     <t>TestScenarioID</t>
+  </si>
+  <si>
+    <t>testCaseType</t>
+  </si>
+  <si>
+    <t>User</t>
+  </si>
+  <si>
+    <t>Role</t>
+  </si>
+  <si>
+    <t>expected</t>
+  </si>
+  <si>
+    <t>Login with spl charac in Username</t>
+  </si>
+  <si>
+    <t>Lmsh@$#athon@gmail.com</t>
+  </si>
+  <si>
+    <t>lmsAug@2026</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>&lt;expected&gt;</t>
+  </si>
+  <si>
+    <t>Empty Username field for signin</t>
+  </si>
+  <si>
+    <t>Empty Password field for signin</t>
+  </si>
+  <si>
+    <t>Lmshackathon@gmail.com</t>
+  </si>
+  <si>
+    <t>Login attempt without selecting any role</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Login Attempt with invalid role</t>
+  </si>
+  <si>
+    <t>lmsA@2020</t>
+  </si>
+  <si>
+    <t>Student</t>
+  </si>
+  <si>
+    <t>Login attempt with wrong password</t>
+  </si>
+  <si>
+    <t>lmsAug@2027</t>
+  </si>
+  <si>
+    <t>Key</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>SearchQuery</t>
+  </si>
+  <si>
+    <t>ExpectedResult</t>
+  </si>
+  <si>
+    <t>validProgram</t>
+  </si>
+  <si>
+    <t>&lt;unique&gt;</t>
+  </si>
+  <si>
+    <t>Playwright automation</t>
+  </si>
+  <si>
+    <t>&lt;created&gt;</t>
+  </si>
+  <si>
+    <t>Program Created Successfully</t>
+  </si>
+  <si>
+    <t>numericProgram</t>
+  </si>
+  <si>
+    <t>12345</t>
+  </si>
+  <si>
+    <t>Invalid numeric program name</t>
+  </si>
+  <si>
+    <t>Name format error</t>
+  </si>
+  <si>
+    <t>existingProgram</t>
+  </si>
+  <si>
+    <t>Java</t>
+  </si>
+  <si>
+    <t>Core Java automation</t>
+  </si>
+  <si>
+    <t>Matching record</t>
+  </si>
+  <si>
+    <t>editProgramName</t>
+  </si>
+  <si>
+    <t>Java Advanced</t>
+  </si>
+  <si>
+    <t>Program Updated</t>
+  </si>
+  <si>
+    <t>editDescription</t>
+  </si>
+  <si>
+    <t>Updated Playwright desc</t>
+  </si>
+  <si>
+    <t>editStatus</t>
+  </si>
+  <si>
+    <t>Inactive</t>
+  </si>
+  <si>
+    <t>deleteProgram</t>
+  </si>
+  <si>
+    <t>JavaDeleteSravanthi</t>
+  </si>
+  <si>
+    <t>Delete test program</t>
+  </si>
+  <si>
+    <t>Program Deleted</t>
+  </si>
+  <si>
+    <t>multiDeleteProgram</t>
+  </si>
+  <si>
+    <t>Bulk Delete</t>
+  </si>
+  <si>
+    <t>Zero results</t>
+  </si>
+  <si>
+    <t>searchByName</t>
+  </si>
+  <si>
+    <t>searchByDescription</t>
+  </si>
+  <si>
+    <t>automation</t>
+  </si>
+  <si>
+    <t>nonExistentProgram</t>
+  </si>
+  <si>
+    <t>NoSuchProgram-987654</t>
+  </si>
+  <si>
+    <t>partialProgramName</t>
+  </si>
+  <si>
+    <t>Jav</t>
+  </si>
+  <si>
+    <t>singleResultProgram</t>
+  </si>
+  <si>
+    <t>Pagination disabled</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -109,16 +257,56 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -126,14 +314,164 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9E2F3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9E2F3"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9E2F3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9E2F3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFD9E2F3"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD9E2F3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9E2F3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9E2F3"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD9E2F3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9E2F3"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD9E2F3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFD9E2F3"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9E2F3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9E2F3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9E2F3"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD9E2F3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9E2F3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFD9E2F3"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9E2F3"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9E2F3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9E2F3"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9E2F3"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9E2F3"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD9E2F3"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -412,57 +750,381 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="41" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
+    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{00C63B44-501C-4008-B50E-28FCAF26870C}"/>
+    <hyperlink ref="C2" r:id="rId2" xr:uid="{C1DDF26E-2F39-4E97-8871-9F4D910B2BBF}"/>
+    <hyperlink ref="B4" r:id="rId3" xr:uid="{F7203CBF-50A5-45DE-9C6C-617904EAD461}"/>
+    <hyperlink ref="C6" r:id="rId4" xr:uid="{4F510F6A-0547-4F24-A175-02BDF50B86F1}"/>
+    <hyperlink ref="C7" r:id="rId5" display="lmsAug@2026" xr:uid="{D20DEC2C-74BB-47BC-B79C-278B22DF23D9}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F15BED11-BCF5-4AB1-8114-513706428888}">
-  <dimension ref="A1:D1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1ADFFFD7-355F-425F-874A-3588F686DED4}">
+  <dimension ref="A1:F14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.7109375" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19" customWidth="1"/>
+    <col min="4" max="4" width="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D1" t="s">
-        <v>4</v>
+    <row r="1" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B6" s="11"/>
+      <c r="C6" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="D6" s="11"/>
+      <c r="E6" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" s="11"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>56</v>
+      </c>
+      <c r="B8" t="s">
+        <v>57</v>
+      </c>
+      <c r="C8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" t="s">
+        <v>57</v>
+      </c>
+      <c r="F8" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C10" s="11"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="B11" s="11"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A12" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" s="11"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B13" s="11"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A14" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="B14" s="14"/>
+      <c r="C14" s="14"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="F14" s="15" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -471,38 +1133,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1ADFFFD7-355F-425F-874A-3588F686DED4}">
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.85546875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A2CCFFE-5A1D-4795-B266-9DD5903277D6}">
   <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -515,36 +1145,36 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="B1" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C1" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="D1" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F1" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="C2">
         <v>42</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="E2">
         <v>15</v>
@@ -552,16 +1182,16 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C3">
         <v>48</v>
       </c>
       <c r="D3" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="E3">
         <v>14</v>
@@ -569,53 +1199,19 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C4">
         <v>56</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="E4">
         <v>20</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9BB8FB4-A4BA-4A8B-A09A-549EA5A8D2A1}">
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="19.7109375" customWidth="1"/>
-    <col min="2" max="2" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.5703125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>